<commit_message>
BOM: gold-contact toggle 100SP1T1B1M2RE (same body and pins)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JAavHVgiwWaG4iqEz4KA1Q
</commit_message>
<xml_diff>
--- a/pcb/carrier/fab/mouser-bom.xlsx
+++ b/pcb/carrier/fab/mouser-bom.xlsx
@@ -482,7 +482,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>100SP1T1B1M2QEH</t>
+          <t>100SP1T1B1M2RE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -500,7 +500,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Toggle SPDT on-on, PCB mount, 1/4-40 bushing, with nuts</t>
+          <t>Toggle SPDT on-on, PCB mount, 1/4-40 bushing, gold contacts</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop JST connectors: footswitch leads solder straight into J1/J2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JAavHVgiwWaG4iqEz4KA1Q
</commit_message>
<xml_diff>
--- a/pcb/carrier/fab/mouser-bom.xlsx
+++ b/pcb/carrier/fab/mouser-bom.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -582,148 +582,73 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>B2B-PH-K-S(LF)(SN)</t>
+          <t>MFR-25FBF52-470R</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>J1 J2</t>
+          <t>R1 R2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2-pin PH header, top entry</t>
+          <t>470 ohm 1/4 W metal film</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PHR-2</t>
+          <t>MFR-25FBF52-100K</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>J1 J2 mates</t>
+          <t>R3 R4</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>PH 2-pin housing</t>
+          <t>100k 1/4 W metal film</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SPH-002T-P0.5S</t>
+          <t>WP59EGW</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Kingbright</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>J1 J2 mates</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
-        <is>
-          <t>PH crimp contact (spares)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>MFR-25FBF52-470R</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Yageo</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>5</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>R1 R2</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>470 ohm 1/4 W metal film</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>MFR-25FBF52-100K</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Yageo</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>5</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>R3 R4</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>100k 1/4 W metal film</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>WP59EGW</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Kingbright</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
         <is>
           <t>5 mm red/green bi-colour LED, 3-lead common cathode</t>
         </is>

</xml_diff>